<commit_message>
feat(production): replace production areas with the recipe's factory [RN-49]
Orders, closes, the plan, imports, the production summary (RN-53), the
dashboard and traceability now show and filter by the factory of the
order's recipe instead of a production area. The production area catalog,
the item's default area, the area column of both imports and the
production.areas.manage permission are removed (migration
RemoveProductionAreas). RN-71/RN-92/RN-93 group by product, date and shift.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/e2e/fixtures/ordenes-con-errores.xlsx
+++ b/frontend/e2e/fixtures/ordenes-con-errores.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,20 +434,15 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>turno</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>turno</t>
+          <t>ubicacion</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
-        <is>
-          <t>ubicacion</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
         <is>
           <t>notas</t>
         </is>
@@ -470,7 +465,6 @@
       <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -489,7 +483,6 @@
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -508,7 +501,6 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>